<commit_message>
convert concentrations to mol/:
</commit_message>
<xml_diff>
--- a/1_Data_inputs/2_Chemical_measurements/ChemistrywTox_MouseMap_042821.xlsx
+++ b/1_Data_inputs/2_Chemical_measurements/ChemistrywTox_MouseMap_042821.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://adminliveunc-my.sharepoint.com/personal/jrchapp3_ad_unc_edu/Documents/Symbolic_regression_github/NIH_Cloud_NOSI/LK_Prelim_Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://adminliveunc-my.sharepoint.com/personal/jrchapp3_ad_unc_edu/Documents/Symbolic_regression_github/NIH_Cloud_NOSI/1_Data_inputs/2_Chemical_measurements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB364041-1732-A845-BB39-F1C1A9B9715B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{DB364041-1732-A845-BB39-F1C1A9B9715B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{524679EE-5C2F-49B2-A817-6C48186DBFB6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E9D93C69-1D32-7543-A0FD-2FB11E5159CA}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{E9D93C69-1D32-7543-A0FD-2FB11E5159CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="4" r:id="rId1"/>
@@ -1425,78 +1425,78 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16299F68-2850-9544-905F-01EB3FA00FDC}">
   <dimension ref="A1:D111"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="14.875" customWidth="1"/>
+    <col min="1" max="1" width="30.59765625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="14.8984375" customWidth="1"/>
     <col min="3" max="4" width="23.5" customWidth="1"/>
-    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.59765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.09765625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.3984375" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="8.8984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.8984375" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="18" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.09765625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="17" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.8984375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.09765625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="16.875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="16.8984375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.59765625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="12" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.09765625" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="20" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.3984375" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="11" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="8" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="6.625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.59765625" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="8.09765625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.59765625" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="13" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.3984375" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="61" max="62" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="63" max="64" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="77" max="78" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="59" max="60" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="61" max="62" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="63" max="64" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="77" max="78" width="5.09765625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="4.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>317</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>318</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
@@ -1552,7 +1552,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>11</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>14</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>15</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>16</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>17</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
@@ -1678,7 +1678,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>19</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>20</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>21</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>24</v>
       </c>
@@ -1762,7 +1762,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>25</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>26</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>27</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>28</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>29</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>30</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>31</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>319</v>
       </c>
@@ -1874,7 +1874,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>320</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>321</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>322</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>323</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>38</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>39</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>307</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>308</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>309</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>310</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>311</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>312</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>46</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>47</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>48</v>
       </c>
@@ -2084,7 +2084,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>49</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>313</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>51</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>52</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>53</v>
       </c>
@@ -2154,7 +2154,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>54</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>55</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>56</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>324</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>59</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>60</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>61</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>62</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>63</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>64</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>65</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>66</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>67</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>68</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>69</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>70</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>73</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>74</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>75</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>76</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>77</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>78</v>
       </c>
@@ -2462,7 +2462,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>314</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>80</v>
       </c>
@@ -2490,7 +2490,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>81</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>82</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>83</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>84</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
         <v>85</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>315</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>87</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>316</v>
       </c>
@@ -2602,7 +2602,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>89</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>90</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
         <v>91</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
         <v>92</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>95</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
         <v>96</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>97</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
         <v>98</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
         <v>99</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
         <v>103</v>
       </c>
@@ -2742,7 +2742,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
         <v>104</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>105</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
         <v>106</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>108</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
         <v>109</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
         <v>110</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
         <v>111</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
         <v>112</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>113</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
         <v>115</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
         <v>116</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
         <v>117</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
         <v>118</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
         <v>119</v>
       </c>
@@ -2938,7 +2938,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
         <v>120</v>
       </c>
@@ -2952,7 +2952,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
         <v>121</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
         <v>122</v>
       </c>
@@ -2980,7 +2980,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
         <v>123</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
         <v>124</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
         <v>127</v>
       </c>
@@ -3022,7 +3022,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
         <v>128</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
         <v>129</v>
       </c>
@@ -3058,87 +3058,87 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E75F7B8F-4A60-B044-93B5-EC9DECD67F96}">
   <dimension ref="A1:N87"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="17.125" customWidth="1"/>
+    <col min="1" max="1" width="30.59765625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="17.09765625" customWidth="1"/>
     <col min="3" max="3" width="23.5" customWidth="1"/>
     <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.8984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.8984375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.5" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.3984375" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="8.8984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.8984375" bestFit="1" customWidth="1"/>
     <col min="28" max="29" width="18" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="21.125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="21.09765625" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="17" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="10.125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="13.8984375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="10.09765625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.8984375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.59765625" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="12" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.09765625" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="20" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13.3984375" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="11" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="8" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="6.59765625" bestFit="1" customWidth="1"/>
     <col min="50" max="50" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="8.09765625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="19.59765625" bestFit="1" customWidth="1"/>
     <col min="59" max="59" width="13" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="14.3984375" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="68" max="69" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="70" max="71" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="84" max="85" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="66" max="67" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="68" max="69" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="70" max="71" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="84" max="85" width="5.09765625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="4.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>130</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
@@ -3226,7 +3226,7 @@
         <v>5.6568542494923796E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>8</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>4.2426406871192847E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
@@ -3314,7 +3314,7 @@
         <v>9.1923881554251172E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>3.5355339059327376E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>11</v>
       </c>
@@ -3402,7 +3402,7 @@
         <v>0.10606601717798211</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>0.12727922061357855</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
@@ -3490,7 +3490,7 @@
         <v>0.12020815280171308</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>14</v>
       </c>
@@ -3534,7 +3534,7 @@
         <v>0.1414213562373095</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>15</v>
       </c>
@@ -3578,7 +3578,7 @@
         <v>0.13435028842544403</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>16</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>9.1923881554251172E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>17</v>
       </c>
@@ -3666,7 +3666,7 @@
         <v>6.3639610306789274E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>0.18384776310850234</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>19</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>6.3639610306789274E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>20</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>2.1213203435596423E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>21</v>
       </c>
@@ -3842,7 +3842,7 @@
         <v>0.16263455967290594</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>22</v>
       </c>
@@ -3886,7 +3886,7 @@
         <v>5.6568542494923796E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
@@ -3930,7 +3930,7 @@
         <v>7.778174593052023E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>24</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>8.4852813742385694E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>25</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>3.5355339059327376E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>26</v>
       </c>
@@ -4062,7 +4062,7 @@
         <v>4.9497474683058325E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>27</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>0.10606601717798211</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>28</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>0.15556349186104046</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>29</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>9.899494936611665E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>30</v>
       </c>
@@ -4238,7 +4238,7 @@
         <v>0.13435028842544403</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>31</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>7.778174593052023E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>32</v>
       </c>
@@ -4326,7 +4326,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>34</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>0.11313708498984759</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>35</v>
       </c>
@@ -4414,7 +4414,7 @@
         <v>6.3639610306789274E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>36</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>6.3639610306789274E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>37</v>
       </c>
@@ -4502,7 +4502,7 @@
         <v>0.10606601717798211</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>38</v>
       </c>
@@ -4546,7 +4546,7 @@
         <v>4.2426406871192847E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>39</v>
       </c>
@@ -4590,7 +4590,7 @@
         <v>2.1213203435596423E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>40</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>4.2426406871192847E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>41</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>42</v>
       </c>
@@ -4722,7 +4722,7 @@
         <v>2.8284271247461898E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>43</v>
       </c>
@@ -4766,7 +4766,7 @@
         <v>4.2426406871192847E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>44</v>
       </c>
@@ -4810,7 +4810,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>45</v>
       </c>
@@ -4854,7 +4854,7 @@
         <v>8.4852813742385694E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>46</v>
       </c>
@@ -4898,7 +4898,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>47</v>
       </c>
@@ -4942,7 +4942,7 @@
         <v>7.0710678118654745E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>48</v>
       </c>
@@ -4986,7 +4986,7 @@
         <v>7.0710678118654745E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>49</v>
       </c>
@@ -5030,7 +5030,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>50</v>
       </c>
@@ -5074,7 +5074,7 @@
         <v>4.9497474683058325E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>51</v>
       </c>
@@ -5118,7 +5118,7 @@
         <v>4.2426406871192847E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>52</v>
       </c>
@@ -5162,7 +5162,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>53</v>
       </c>
@@ -5206,7 +5206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>54</v>
       </c>
@@ -5250,7 +5250,7 @@
         <v>7.0710678118654745E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>55</v>
       </c>
@@ -5294,7 +5294,7 @@
         <v>2.1213203435596423E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>56</v>
       </c>
@@ -5338,7 +5338,7 @@
         <v>2.8284271247461898E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>57</v>
       </c>
@@ -5382,7 +5382,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>59</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>60</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>61</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>62</v>
       </c>
@@ -5558,7 +5558,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>63</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>64</v>
       </c>
@@ -5646,7 +5646,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>65</v>
       </c>
@@ -5690,7 +5690,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>66</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>67</v>
       </c>
@@ -5778,7 +5778,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>68</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>0.35355339059327373</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>69</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>0.17677669529663687</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>70</v>
       </c>
@@ -5910,7 +5910,7 @@
         <v>0.8987327188881018</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>73</v>
       </c>
@@ -5954,7 +5954,7 @@
         <v>3.1112698372208088E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>74</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>1.936058366888767</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>75</v>
       </c>
@@ -6042,7 +6042,7 @@
         <v>2.1920310216782972E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>76</v>
       </c>
@@ -6086,7 +6086,7 @@
         <v>3.3234018715767734E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>77</v>
       </c>
@@ -6130,7 +6130,7 @@
         <v>2.8284271247461898E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>78</v>
       </c>
@@ -6174,7 +6174,7 @@
         <v>0.26870057685088805</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>79</v>
       </c>
@@ -6218,7 +6218,7 @@
         <v>0.55932146391855908</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>80</v>
       </c>
@@ -6262,7 +6262,7 @@
         <v>0.21991020894901625</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>81</v>
       </c>
@@ -6306,7 +6306,7 @@
         <v>3.3234018715767734E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>82</v>
       </c>
@@ -6350,7 +6350,7 @@
         <v>0.58194888091652852</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>83</v>
       </c>
@@ -6394,7 +6394,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>84</v>
       </c>
@@ -6438,7 +6438,7 @@
         <v>0.19940411229460636</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
         <v>85</v>
       </c>
@@ -6482,7 +6482,7 @@
         <v>2.9698484809834995E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>86</v>
       </c>
@@ -6526,7 +6526,7 @@
         <v>70.710678118654741</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>87</v>
       </c>
@@ -6570,7 +6570,7 @@
         <v>3.1819805153394637E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>88</v>
       </c>
@@ -6614,7 +6614,7 @@
         <v>3.3941125496954276</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>89</v>
       </c>
@@ -6658,7 +6658,7 @@
         <v>1.4142135623730949E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>90</v>
       </c>
@@ -6702,7 +6702,7 @@
         <v>4.2426406871192847E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
         <v>91</v>
       </c>
@@ -6746,7 +6746,7 @@
         <v>9.616652224137047E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
         <v>92</v>
       </c>
@@ -6790,7 +6790,7 @@
         <v>9.9702056147303198E-3</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>95</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>5.12652416360247E-4</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
         <v>96</v>
       </c>
@@ -6878,7 +6878,7 @@
         <v>5.550788232314397E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>97</v>
       </c>
@@ -6922,7 +6922,7 @@
         <v>5.3033008588990866E-4</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
         <v>98</v>
       </c>
@@ -6974,24 +6974,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3778C7D-8528-024D-BB3E-C7B335D16723}">
   <dimension ref="A1:O71"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.375" customWidth="1"/>
-    <col min="2" max="3" width="23.625" customWidth="1"/>
-    <col min="4" max="4" width="27.875" customWidth="1"/>
-    <col min="5" max="5" width="29.375" customWidth="1"/>
-    <col min="6" max="7" width="17.625" customWidth="1"/>
+    <col min="1" max="1" width="29.3984375" customWidth="1"/>
+    <col min="2" max="3" width="23.59765625" customWidth="1"/>
+    <col min="4" max="4" width="27.8984375" customWidth="1"/>
+    <col min="5" max="5" width="29.3984375" customWidth="1"/>
+    <col min="6" max="7" width="17.59765625" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="19.375" customWidth="1"/>
+    <col min="9" max="9" width="19.3984375" customWidth="1"/>
     <col min="10" max="10" width="16.5" customWidth="1"/>
-    <col min="11" max="11" width="19.375" customWidth="1"/>
+    <col min="11" max="11" width="19.3984375" customWidth="1"/>
     <col min="12" max="12" width="26.5" customWidth="1"/>
-    <col min="13" max="13" width="19.375" customWidth="1"/>
-    <col min="14" max="14" width="16.125" customWidth="1"/>
-    <col min="15" max="15" width="14.125" customWidth="1"/>
+    <col min="13" max="13" width="19.3984375" customWidth="1"/>
+    <col min="14" max="14" width="16.09765625" customWidth="1"/>
+    <col min="15" max="15" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>143</v>
       </c>
@@ -7038,7 +7038,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>157</v>
       </c>
@@ -7085,7 +7085,7 @@
         <v>3.1789999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>157</v>
       </c>
@@ -7132,7 +7132,7 @@
         <v>4.4740000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>157</v>
       </c>
@@ -7179,7 +7179,7 @@
         <v>3.4950000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>157</v>
       </c>
@@ -7210,7 +7210,7 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>157</v>
       </c>
@@ -7257,7 +7257,7 @@
         <v>3.847</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>157</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>132</v>
       </c>
@@ -7351,7 +7351,7 @@
         <v>3.6040000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>132</v>
       </c>
@@ -7398,7 +7398,7 @@
         <v>3.6669999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>132</v>
       </c>
@@ -7445,7 +7445,7 @@
         <v>3.806</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>132</v>
       </c>
@@ -7492,7 +7492,7 @@
         <v>3.8879999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>132</v>
       </c>
@@ -7539,7 +7539,7 @@
         <v>4.1429999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>132</v>
       </c>
@@ -7586,7 +7586,7 @@
         <v>5.6070000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>133</v>
       </c>
@@ -7633,7 +7633,7 @@
         <v>3.9380000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>133</v>
       </c>
@@ -7680,7 +7680,7 @@
         <v>3.867</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>133</v>
       </c>
@@ -7727,7 +7727,7 @@
         <v>3.9780000000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>133</v>
       </c>
@@ -7774,7 +7774,7 @@
         <v>4.0350000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>133</v>
       </c>
@@ -7821,7 +7821,7 @@
         <v>2.653</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>133</v>
       </c>
@@ -7868,7 +7868,7 @@
         <v>3.012</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>134</v>
       </c>
@@ -7915,7 +7915,7 @@
         <v>3.875</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>134</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>4.2030000000000003</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>134</v>
       </c>
@@ -8009,7 +8009,7 @@
         <v>3.9649999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>134</v>
       </c>
@@ -8056,7 +8056,7 @@
         <v>2.7109999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>134</v>
       </c>
@@ -8103,7 +8103,7 @@
         <v>3.1219999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>134</v>
       </c>
@@ -8150,7 +8150,7 @@
         <v>3.3889999999999998</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>135</v>
       </c>
@@ -8197,7 +8197,7 @@
         <v>3.3730000000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>135</v>
       </c>
@@ -8244,7 +8244,7 @@
         <v>3.6019999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>135</v>
       </c>
@@ -8291,7 +8291,7 @@
         <v>4.867</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>135</v>
       </c>
@@ -8338,7 +8338,7 @@
         <v>3.8439999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>135</v>
       </c>
@@ -8385,7 +8385,7 @@
         <v>3.8719999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>135</v>
       </c>
@@ -8432,7 +8432,7 @@
         <v>4.0620000000000003</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>136</v>
       </c>
@@ -8479,7 +8479,7 @@
         <v>3.52</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>136</v>
       </c>
@@ -8526,7 +8526,7 @@
         <v>3.6040000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>136</v>
       </c>
@@ -8573,7 +8573,7 @@
         <v>3.7210000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>136</v>
       </c>
@@ -8620,7 +8620,7 @@
         <v>3.95</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
         <v>136</v>
       </c>
@@ -8667,7 +8667,7 @@
         <v>4.1619999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
         <v>136</v>
       </c>
@@ -8714,7 +8714,7 @@
         <v>4.226</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
         <v>137</v>
       </c>
@@ -8761,7 +8761,7 @@
         <v>4.0979999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
         <v>137</v>
       </c>
@@ -8808,7 +8808,7 @@
         <v>4.1769999999999996</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
         <v>137</v>
       </c>
@@ -8855,7 +8855,7 @@
         <v>2.794</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>137</v>
       </c>
@@ -8902,7 +8902,7 @@
         <v>2.9740000000000002</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
         <v>137</v>
       </c>
@@ -8949,7 +8949,7 @@
         <v>3.137</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
         <v>137</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>3.2189999999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
         <v>138</v>
       </c>
@@ -9043,7 +9043,7 @@
         <v>5.1280000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
         <v>138</v>
       </c>
@@ -9090,7 +9090,7 @@
         <v>4.2880000000000003</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
         <v>138</v>
       </c>
@@ -9137,7 +9137,7 @@
         <v>2.726</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
         <v>138</v>
       </c>
@@ -9184,7 +9184,7 @@
         <v>2.988</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
         <v>138</v>
       </c>
@@ -9231,7 +9231,7 @@
         <v>3.1520000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
         <v>138</v>
       </c>
@@ -9276,7 +9276,7 @@
         <v>4.8860000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>139</v>
       </c>
@@ -9323,7 +9323,7 @@
         <v>3.3959999999999999</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
         <v>139</v>
       </c>
@@ -9370,7 +9370,7 @@
         <v>3.4580000000000002</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
         <v>139</v>
       </c>
@@ -9417,7 +9417,7 @@
         <v>3.673</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="8" t="s">
         <v>139</v>
       </c>
@@ -9464,7 +9464,7 @@
         <v>3.7949999999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>139</v>
       </c>
@@ -9511,7 +9511,7 @@
         <v>3.9980000000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
         <v>139</v>
       </c>
@@ -9558,7 +9558,7 @@
         <v>3.7309999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
         <v>140</v>
       </c>
@@ -9605,7 +9605,7 @@
         <v>2.7240000000000002</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
         <v>140</v>
       </c>
@@ -9652,7 +9652,7 @@
         <v>2.923</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
         <v>140</v>
       </c>
@@ -9699,7 +9699,7 @@
         <v>3.1829999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
         <v>140</v>
       </c>
@@ -9746,7 +9746,7 @@
         <v>3.3039999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
         <v>140</v>
       </c>
@@ -9793,7 +9793,7 @@
         <v>3.448</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="8" t="s">
         <v>140</v>
       </c>
@@ -9840,7 +9840,7 @@
         <v>3.694</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="8" t="s">
         <v>141</v>
       </c>
@@ -9887,7 +9887,7 @@
         <v>3.44</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
         <v>141</v>
       </c>
@@ -9934,7 +9934,7 @@
         <v>3.2570000000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="8" t="s">
         <v>141</v>
       </c>
@@ -9981,7 +9981,7 @@
         <v>2.6230000000000002</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="8" t="s">
         <v>141</v>
       </c>
@@ -10028,7 +10028,7 @@
         <v>2.9449999999999998</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="8" t="s">
         <v>141</v>
       </c>
@@ -10075,7 +10075,7 @@
         <v>3.2879999999999998</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="8" t="s">
         <v>141</v>
       </c>
@@ -10122,7 +10122,7 @@
         <v>3.3719999999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
         <v>231</v>
       </c>
@@ -10169,7 +10169,7 @@
         <v>2.8919999999999999</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="8" t="s">
         <v>231</v>
       </c>
@@ -10216,7 +10216,7 @@
         <v>3.18</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="8" t="s">
         <v>231</v>
       </c>
@@ -10263,7 +10263,7 @@
         <v>3.3460000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="8" t="s">
         <v>231</v>
       </c>
@@ -10321,24 +10321,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53860B46-7720-1543-939B-0DB3E7608629}">
   <dimension ref="A1:O71"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.375" customWidth="1"/>
-    <col min="2" max="3" width="23.625" customWidth="1"/>
-    <col min="4" max="4" width="27.875" customWidth="1"/>
-    <col min="5" max="5" width="29.375" customWidth="1"/>
-    <col min="6" max="7" width="17.625" customWidth="1"/>
+    <col min="1" max="1" width="29.3984375" customWidth="1"/>
+    <col min="2" max="3" width="23.59765625" customWidth="1"/>
+    <col min="4" max="4" width="27.8984375" customWidth="1"/>
+    <col min="5" max="5" width="29.3984375" customWidth="1"/>
+    <col min="6" max="7" width="17.59765625" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="19.375" customWidth="1"/>
+    <col min="9" max="9" width="19.3984375" customWidth="1"/>
     <col min="10" max="10" width="16.5" customWidth="1"/>
-    <col min="11" max="11" width="19.375" customWidth="1"/>
+    <col min="11" max="11" width="19.3984375" customWidth="1"/>
     <col min="12" max="12" width="26.5" customWidth="1"/>
-    <col min="13" max="13" width="19.375" customWidth="1"/>
-    <col min="14" max="14" width="16.125" customWidth="1"/>
-    <col min="15" max="15" width="14.125" customWidth="1"/>
+    <col min="13" max="13" width="19.3984375" customWidth="1"/>
+    <col min="14" max="14" width="16.09765625" customWidth="1"/>
+    <col min="15" max="15" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>143</v>
       </c>
@@ -10385,7 +10385,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>157</v>
       </c>
@@ -10432,7 +10432,7 @@
         <v>3.5750000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>157</v>
       </c>
@@ -10479,7 +10479,7 @@
         <v>2.6880000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>157</v>
       </c>
@@ -10526,7 +10526,7 @@
         <v>3.153</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>157</v>
       </c>
@@ -10573,7 +10573,7 @@
         <v>3.4020000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>157</v>
       </c>
@@ -10620,7 +10620,7 @@
         <v>3.508</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>157</v>
       </c>
@@ -10667,7 +10667,7 @@
         <v>3.7170000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>132</v>
       </c>
@@ -10714,7 +10714,7 @@
         <v>5.03</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>132</v>
       </c>
@@ -10761,7 +10761,7 @@
         <v>5.3769999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>132</v>
       </c>
@@ -10808,7 +10808,7 @@
         <v>5.891</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>132</v>
       </c>
@@ -10855,7 +10855,7 @@
         <v>3.2719999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>132</v>
       </c>
@@ -10902,7 +10902,7 @@
         <v>3.407</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>132</v>
       </c>
@@ -10949,7 +10949,7 @@
         <v>3.6659999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>133</v>
       </c>
@@ -10996,7 +10996,7 @@
         <v>4.3730000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>133</v>
       </c>
@@ -11043,7 +11043,7 @@
         <v>4.4470000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>133</v>
       </c>
@@ -11090,7 +11090,7 @@
         <v>4.5439999999999996</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>133</v>
       </c>
@@ -11137,7 +11137,7 @@
         <v>4.3819999999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>133</v>
       </c>
@@ -11184,7 +11184,7 @@
         <v>2.8260000000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>133</v>
       </c>
@@ -11231,7 +11231,7 @@
         <v>3.258</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>134</v>
       </c>
@@ -11278,7 +11278,7 @@
         <v>3.0169999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>134</v>
       </c>
@@ -11325,7 +11325,7 @@
         <v>3.26</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>134</v>
       </c>
@@ -11372,7 +11372,7 @@
         <v>3.2759999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>134</v>
       </c>
@@ -11419,7 +11419,7 @@
         <v>3.4830000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>134</v>
       </c>
@@ -11466,7 +11466,7 @@
         <v>3.6589999999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>134</v>
       </c>
@@ -11513,7 +11513,7 @@
         <v>3.8580000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>135</v>
       </c>
@@ -11560,7 +11560,7 @@
         <v>3.472</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>135</v>
       </c>
@@ -11607,7 +11607,7 @@
         <v>3.637</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>135</v>
       </c>
@@ -11654,7 +11654,7 @@
         <v>3.7669999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>135</v>
       </c>
@@ -11701,7 +11701,7 @@
         <v>3.9710000000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>135</v>
       </c>
@@ -11748,7 +11748,7 @@
         <v>4.1529999999999996</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>135</v>
       </c>
@@ -11795,7 +11795,7 @@
         <v>5.4630000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>136</v>
       </c>
@@ -11842,7 +11842,7 @@
         <v>3.996</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>136</v>
       </c>
@@ -11889,7 +11889,7 @@
         <v>4.3040000000000003</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>136</v>
       </c>
@@ -11918,7 +11918,7 @@
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>136</v>
       </c>
@@ -11965,7 +11965,7 @@
         <v>4.2699999999999996</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
         <v>136</v>
       </c>
@@ -12012,7 +12012,7 @@
         <v>2.8039999999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
         <v>136</v>
       </c>
@@ -12059,7 +12059,7 @@
         <v>3.0489999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
         <v>137</v>
       </c>
@@ -12106,7 +12106,7 @@
         <v>5.5620000000000003</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
         <v>137</v>
       </c>
@@ -12153,7 +12153,7 @@
         <v>6.29</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
         <v>137</v>
       </c>
@@ -12200,7 +12200,7 @@
         <v>3.2559999999999998</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>137</v>
       </c>
@@ -12247,7 +12247,7 @@
         <v>3.4390000000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
         <v>137</v>
       </c>
@@ -12294,7 +12294,7 @@
         <v>3.6160000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
         <v>137</v>
       </c>
@@ -12341,7 +12341,7 @@
         <v>3.7170000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
         <v>138</v>
       </c>
@@ -12388,7 +12388,7 @@
         <v>3.3140000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
         <v>138</v>
       </c>
@@ -12435,7 +12435,7 @@
         <v>3.5379999999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
         <v>138</v>
       </c>
@@ -12482,7 +12482,7 @@
         <v>3.6480000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
         <v>138</v>
       </c>
@@ -12529,7 +12529,7 @@
         <v>3.8450000000000002</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
         <v>138</v>
       </c>
@@ -12576,7 +12576,7 @@
         <v>4.0869999999999997</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
         <v>138</v>
       </c>
@@ -12623,7 +12623,7 @@
         <v>4.2270000000000003</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>139</v>
       </c>
@@ -12670,7 +12670,7 @@
         <v>4.0279999999999996</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
         <v>139</v>
       </c>
@@ -12717,7 +12717,7 @@
         <v>3.6539999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
         <v>139</v>
       </c>
@@ -12764,7 +12764,7 @@
         <v>3.617</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="8" t="s">
         <v>139</v>
       </c>
@@ -12811,7 +12811,7 @@
         <v>3.82</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>139</v>
       </c>
@@ -12858,7 +12858,7 @@
         <v>3.9969999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
         <v>139</v>
       </c>
@@ -12905,7 +12905,7 @@
         <v>4.1989999999999998</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
         <v>140</v>
       </c>
@@ -12952,7 +12952,7 @@
         <v>3.8889999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
         <v>140</v>
       </c>
@@ -12999,7 +12999,7 @@
         <v>4.0709999999999997</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
         <v>140</v>
       </c>
@@ -13046,7 +13046,7 @@
         <v>4.29</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
         <v>140</v>
       </c>
@@ -13093,7 +13093,7 @@
         <v>4.367</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
         <v>140</v>
       </c>
@@ -13140,7 +13140,7 @@
         <v>5.3659999999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="8" t="s">
         <v>140</v>
       </c>
@@ -13187,7 +13187,7 @@
         <v>4.1059999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="8" t="s">
         <v>141</v>
       </c>
@@ -13234,7 +13234,7 @@
         <v>3.677</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
         <v>141</v>
       </c>
@@ -13281,7 +13281,7 @@
         <v>3.8279999999999998</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="8" t="s">
         <v>141</v>
       </c>
@@ -13328,7 +13328,7 @@
         <v>3.9550000000000001</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="8" t="s">
         <v>141</v>
       </c>
@@ -13375,7 +13375,7 @@
         <v>3.605</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="8" t="s">
         <v>141</v>
       </c>
@@ -13422,7 +13422,7 @@
         <v>3.077</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="8" t="s">
         <v>141</v>
       </c>
@@ -13469,7 +13469,7 @@
         <v>3.3730000000000002</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
         <v>231</v>
       </c>
@@ -13516,7 +13516,7 @@
         <v>3.9849999999999999</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="8" t="s">
         <v>231</v>
       </c>
@@ -13563,7 +13563,7 @@
         <v>3.8980000000000001</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="8" t="s">
         <v>231</v>
       </c>
@@ -13610,7 +13610,7 @@
         <v>3.6930000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="8" t="s">
         <v>231</v>
       </c>
@@ -13663,6 +13663,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A8DF4565409F7A498078360796F26CA9" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d9fe6ba3ad0296993fdf9ca86fb8ec6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="13928eb9-0d8a-4018-8962-fa9e89967672" xmlns:ns3="d960e8a8-69e2-40a4-bb78-08ff18f8bb2f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="84c00418da9684fb2e9f40c453441992" ns2:_="" ns3:_="">
     <xsd:import namespace="13928eb9-0d8a-4018-8962-fa9e89967672"/>
@@ -13917,16 +13926,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C7EE5A2-8461-4909-A45F-0A6C43DF2417}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{209E5E74-AAAA-4AAD-832B-22F4FC51D717}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13943,12 +13951,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C7EE5A2-8461-4909-A45F-0A6C43DF2417}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>